<commit_message>
daily auto-refresh 2026-08-20 13:06
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K309"/>
+  <dimension ref="A1:K310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11869,6 +11869,43 @@
         <v>109</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>3</v>
+      </c>
+      <c r="C310" t="n">
+        <v>6</v>
+      </c>
+      <c r="D310" t="n">
+        <v>0</v>
+      </c>
+      <c r="E310" t="n">
+        <v>0</v>
+      </c>
+      <c r="F310" t="n">
+        <v>2</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="n">
+        <v>0</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-21 13:02
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K310"/>
+  <dimension ref="A1:K311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11654,7 +11654,7 @@
         </is>
       </c>
       <c r="B304" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C304" t="n">
         <v>120</v>
@@ -11681,7 +11681,7 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="305">
@@ -11876,34 +11876,71 @@
         </is>
       </c>
       <c r="B310" t="n">
+        <v>10</v>
+      </c>
+      <c r="C310" t="n">
+        <v>12</v>
+      </c>
+      <c r="D310" t="n">
+        <v>0</v>
+      </c>
+      <c r="E310" t="n">
+        <v>0</v>
+      </c>
+      <c r="F310" t="n">
+        <v>8</v>
+      </c>
+      <c r="G310" t="n">
+        <v>1</v>
+      </c>
+      <c r="H310" t="n">
+        <v>0</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>5</v>
+      </c>
+      <c r="C311" t="n">
         <v>3</v>
       </c>
-      <c r="C310" t="n">
-        <v>6</v>
-      </c>
-      <c r="D310" t="n">
-        <v>0</v>
-      </c>
-      <c r="E310" t="n">
-        <v>0</v>
-      </c>
-      <c r="F310" t="n">
-        <v>2</v>
-      </c>
-      <c r="G310" t="n">
-        <v>0</v>
-      </c>
-      <c r="H310" t="n">
-        <v>0</v>
-      </c>
-      <c r="I310" t="n">
-        <v>0</v>
-      </c>
-      <c r="J310" t="n">
-        <v>0</v>
-      </c>
-      <c r="K310" t="n">
-        <v>11</v>
+      <c r="D311" t="n">
+        <v>0</v>
+      </c>
+      <c r="E311" t="n">
+        <v>0</v>
+      </c>
+      <c r="F311" t="n">
+        <v>1</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" t="n">
+        <v>0</v>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-24 11:00
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K311"/>
+  <dimension ref="A1:K314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11913,34 +11913,145 @@
         </is>
       </c>
       <c r="B311" t="n">
+        <v>18</v>
+      </c>
+      <c r="C311" t="n">
+        <v>10</v>
+      </c>
+      <c r="D311" t="n">
+        <v>0</v>
+      </c>
+      <c r="E311" t="n">
+        <v>1</v>
+      </c>
+      <c r="F311" t="n">
+        <v>4</v>
+      </c>
+      <c r="G311" t="n">
+        <v>1</v>
+      </c>
+      <c r="H311" t="n">
+        <v>0</v>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>14</v>
+      </c>
+      <c r="C312" t="n">
+        <v>19</v>
+      </c>
+      <c r="D312" t="n">
+        <v>0</v>
+      </c>
+      <c r="E312" t="n">
+        <v>0</v>
+      </c>
+      <c r="F312" t="n">
+        <v>10</v>
+      </c>
+      <c r="G312" t="n">
+        <v>2</v>
+      </c>
+      <c r="H312" t="n">
+        <v>1</v>
+      </c>
+      <c r="I312" t="n">
+        <v>0</v>
+      </c>
+      <c r="J312" t="n">
+        <v>0</v>
+      </c>
+      <c r="K312" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>9</v>
+      </c>
+      <c r="C313" t="n">
+        <v>7</v>
+      </c>
+      <c r="D313" t="n">
+        <v>0</v>
+      </c>
+      <c r="E313" t="n">
+        <v>0</v>
+      </c>
+      <c r="F313" t="n">
         <v>5</v>
       </c>
-      <c r="C311" t="n">
-        <v>3</v>
-      </c>
-      <c r="D311" t="n">
-        <v>0</v>
-      </c>
-      <c r="E311" t="n">
-        <v>0</v>
-      </c>
-      <c r="F311" t="n">
-        <v>1</v>
-      </c>
-      <c r="G311" t="n">
-        <v>0</v>
-      </c>
-      <c r="H311" t="n">
-        <v>0</v>
-      </c>
-      <c r="I311" t="n">
-        <v>0</v>
-      </c>
-      <c r="J311" t="n">
-        <v>0</v>
-      </c>
-      <c r="K311" t="n">
-        <v>9</v>
+      <c r="G313" t="n">
+        <v>2</v>
+      </c>
+      <c r="H313" t="n">
+        <v>0</v>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
+        <v>0</v>
+      </c>
+      <c r="K313" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>0</v>
+      </c>
+      <c r="C314" t="n">
+        <v>1</v>
+      </c>
+      <c r="D314" t="n">
+        <v>0</v>
+      </c>
+      <c r="E314" t="n">
+        <v>0</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" t="n">
+        <v>0</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-01 17:00
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K321"/>
+  <dimension ref="A1:L321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Total units</t>
         </is>
       </c>
@@ -507,6 +512,9 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -544,6 +552,9 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
         <v>3</v>
       </c>
     </row>
@@ -581,6 +592,9 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -618,6 +632,9 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -655,6 +672,9 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
         <v>17</v>
       </c>
     </row>
@@ -692,6 +712,9 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
         <v>3</v>
       </c>
     </row>
@@ -729,6 +752,9 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -766,6 +792,9 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
         <v>6</v>
       </c>
     </row>
@@ -803,6 +832,9 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
         <v>4</v>
       </c>
     </row>
@@ -840,6 +872,9 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -877,6 +912,9 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
         <v>5</v>
       </c>
     </row>
@@ -914,6 +952,9 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
         <v>6</v>
       </c>
     </row>
@@ -951,6 +992,9 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
         <v>9</v>
       </c>
     </row>
@@ -988,6 +1032,9 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1025,6 +1072,9 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1062,6 +1112,9 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1099,6 +1152,9 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1136,6 +1192,9 @@
         <v>0</v>
       </c>
       <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
         <v>28</v>
       </c>
     </row>
@@ -1173,6 +1232,9 @@
         <v>0</v>
       </c>
       <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
         <v>26</v>
       </c>
     </row>
@@ -1210,6 +1272,9 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1247,6 +1312,9 @@
         <v>0</v>
       </c>
       <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
         <v>29</v>
       </c>
     </row>
@@ -1284,6 +1352,9 @@
         <v>0</v>
       </c>
       <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
         <v>29</v>
       </c>
     </row>
@@ -1321,6 +1392,9 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1358,6 +1432,9 @@
         <v>0</v>
       </c>
       <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1395,6 +1472,9 @@
         <v>0</v>
       </c>
       <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1432,6 +1512,9 @@
         <v>0</v>
       </c>
       <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1469,6 +1552,9 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1506,6 +1592,9 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
         <v>14</v>
       </c>
     </row>
@@ -1543,6 +1632,9 @@
         <v>0</v>
       </c>
       <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
         <v>27</v>
       </c>
     </row>
@@ -1580,6 +1672,9 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1617,6 +1712,9 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1654,6 +1752,9 @@
         <v>0</v>
       </c>
       <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1691,6 +1792,9 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1728,6 +1832,9 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1765,6 +1872,9 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
         <v>23</v>
       </c>
     </row>
@@ -1802,6 +1912,9 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1839,6 +1952,9 @@
         <v>0</v>
       </c>
       <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1876,6 +1992,9 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1913,6 +2032,9 @@
         <v>0</v>
       </c>
       <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1950,6 +2072,9 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1987,6 +2112,9 @@
         <v>0</v>
       </c>
       <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2024,6 +2152,9 @@
         <v>0</v>
       </c>
       <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2061,6 +2192,9 @@
         <v>0</v>
       </c>
       <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2098,6 +2232,9 @@
         <v>0</v>
       </c>
       <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2135,6 +2272,9 @@
         <v>0</v>
       </c>
       <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2172,6 +2312,9 @@
         <v>0</v>
       </c>
       <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2209,6 +2352,9 @@
         <v>0</v>
       </c>
       <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="n">
         <v>49</v>
       </c>
     </row>
@@ -2246,6 +2392,9 @@
         <v>0</v>
       </c>
       <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2283,6 +2432,9 @@
         <v>0</v>
       </c>
       <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2320,6 +2472,9 @@
         <v>0</v>
       </c>
       <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2357,6 +2512,9 @@
         <v>0</v>
       </c>
       <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2394,6 +2552,9 @@
         <v>0</v>
       </c>
       <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="n">
         <v>31</v>
       </c>
     </row>
@@ -2431,6 +2592,9 @@
         <v>0</v>
       </c>
       <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2468,6 +2632,9 @@
         <v>0</v>
       </c>
       <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2505,6 +2672,9 @@
         <v>0</v>
       </c>
       <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="n">
         <v>70</v>
       </c>
     </row>
@@ -2542,6 +2712,9 @@
         <v>0</v>
       </c>
       <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="n">
         <v>26</v>
       </c>
     </row>
@@ -2579,6 +2752,9 @@
         <v>0</v>
       </c>
       <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="n">
         <v>44</v>
       </c>
     </row>
@@ -2616,6 +2792,9 @@
         <v>0</v>
       </c>
       <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2653,6 +2832,9 @@
         <v>0</v>
       </c>
       <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="n">
         <v>39</v>
       </c>
     </row>
@@ -2690,6 +2872,9 @@
         <v>0</v>
       </c>
       <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="n">
         <v>27</v>
       </c>
     </row>
@@ -2727,6 +2912,9 @@
         <v>0</v>
       </c>
       <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2764,6 +2952,9 @@
         <v>0</v>
       </c>
       <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2801,6 +2992,9 @@
         <v>0</v>
       </c>
       <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2838,6 +3032,9 @@
         <v>0</v>
       </c>
       <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="n">
         <v>41</v>
       </c>
     </row>
@@ -2875,6 +3072,9 @@
         <v>0</v>
       </c>
       <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2912,6 +3112,9 @@
         <v>0</v>
       </c>
       <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="n">
         <v>38</v>
       </c>
     </row>
@@ -2949,6 +3152,9 @@
         <v>0</v>
       </c>
       <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="n">
         <v>29</v>
       </c>
     </row>
@@ -2986,6 +3192,9 @@
         <v>0</v>
       </c>
       <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3023,6 +3232,9 @@
         <v>0</v>
       </c>
       <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="n">
         <v>29</v>
       </c>
     </row>
@@ -3060,6 +3272,9 @@
         <v>0</v>
       </c>
       <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="n">
         <v>35</v>
       </c>
     </row>
@@ -3097,6 +3312,9 @@
         <v>0</v>
       </c>
       <c r="K72" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" t="n">
         <v>35</v>
       </c>
     </row>
@@ -3134,6 +3352,9 @@
         <v>0</v>
       </c>
       <c r="K73" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3171,6 +3392,9 @@
         <v>0</v>
       </c>
       <c r="K74" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" t="n">
         <v>46</v>
       </c>
     </row>
@@ -3208,6 +3432,9 @@
         <v>0</v>
       </c>
       <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3245,6 +3472,9 @@
         <v>0</v>
       </c>
       <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3282,6 +3512,9 @@
         <v>0</v>
       </c>
       <c r="K77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3319,6 +3552,9 @@
         <v>0</v>
       </c>
       <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
         <v>57</v>
       </c>
     </row>
@@ -3356,6 +3592,9 @@
         <v>0</v>
       </c>
       <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3393,6 +3632,9 @@
         <v>0</v>
       </c>
       <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3430,6 +3672,9 @@
         <v>0</v>
       </c>
       <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3467,6 +3712,9 @@
         <v>0</v>
       </c>
       <c r="K82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" t="n">
         <v>22</v>
       </c>
     </row>
@@ -3504,6 +3752,9 @@
         <v>0</v>
       </c>
       <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3541,6 +3792,9 @@
         <v>0</v>
       </c>
       <c r="K84" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3578,6 +3832,9 @@
         <v>0</v>
       </c>
       <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3615,6 +3872,9 @@
         <v>0</v>
       </c>
       <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="n">
         <v>36</v>
       </c>
     </row>
@@ -3652,6 +3912,9 @@
         <v>0</v>
       </c>
       <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3689,6 +3952,9 @@
         <v>0</v>
       </c>
       <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="n">
         <v>23</v>
       </c>
     </row>
@@ -3726,6 +3992,9 @@
         <v>0</v>
       </c>
       <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3763,6 +4032,9 @@
         <v>0</v>
       </c>
       <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="n">
         <v>13</v>
       </c>
     </row>
@@ -3800,6 +4072,9 @@
         <v>0</v>
       </c>
       <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="n">
         <v>39</v>
       </c>
     </row>
@@ -3837,6 +4112,9 @@
         <v>0</v>
       </c>
       <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="n">
         <v>28</v>
       </c>
     </row>
@@ -3874,6 +4152,9 @@
         <v>0</v>
       </c>
       <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3911,6 +4192,9 @@
         <v>0</v>
       </c>
       <c r="K94" t="n">
+        <v>0</v>
+      </c>
+      <c r="L94" t="n">
         <v>46</v>
       </c>
     </row>
@@ -3948,6 +4232,9 @@
         <v>0</v>
       </c>
       <c r="K95" t="n">
+        <v>0</v>
+      </c>
+      <c r="L95" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3985,6 +4272,9 @@
         <v>0</v>
       </c>
       <c r="K96" t="n">
+        <v>0</v>
+      </c>
+      <c r="L96" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4022,6 +4312,9 @@
         <v>0</v>
       </c>
       <c r="K97" t="n">
+        <v>0</v>
+      </c>
+      <c r="L97" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4059,6 +4352,9 @@
         <v>0</v>
       </c>
       <c r="K98" t="n">
+        <v>0</v>
+      </c>
+      <c r="L98" t="n">
         <v>21</v>
       </c>
     </row>
@@ -4096,6 +4392,9 @@
         <v>0</v>
       </c>
       <c r="K99" t="n">
+        <v>0</v>
+      </c>
+      <c r="L99" t="n">
         <v>23</v>
       </c>
     </row>
@@ -4133,6 +4432,9 @@
         <v>0</v>
       </c>
       <c r="K100" t="n">
+        <v>0</v>
+      </c>
+      <c r="L100" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4170,6 +4472,9 @@
         <v>0</v>
       </c>
       <c r="K101" t="n">
+        <v>0</v>
+      </c>
+      <c r="L101" t="n">
         <v>42</v>
       </c>
     </row>
@@ -4207,6 +4512,9 @@
         <v>0</v>
       </c>
       <c r="K102" t="n">
+        <v>0</v>
+      </c>
+      <c r="L102" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4244,6 +4552,9 @@
         <v>0</v>
       </c>
       <c r="K103" t="n">
+        <v>0</v>
+      </c>
+      <c r="L103" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4281,6 +4592,9 @@
         <v>0</v>
       </c>
       <c r="K104" t="n">
+        <v>0</v>
+      </c>
+      <c r="L104" t="n">
         <v>53</v>
       </c>
     </row>
@@ -4318,6 +4632,9 @@
         <v>0</v>
       </c>
       <c r="K105" t="n">
+        <v>0</v>
+      </c>
+      <c r="L105" t="n">
         <v>29</v>
       </c>
     </row>
@@ -4355,6 +4672,9 @@
         <v>0</v>
       </c>
       <c r="K106" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4392,6 +4712,9 @@
         <v>0</v>
       </c>
       <c r="K107" t="n">
+        <v>0</v>
+      </c>
+      <c r="L107" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4429,6 +4752,9 @@
         <v>0</v>
       </c>
       <c r="K108" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4466,6 +4792,9 @@
         <v>0</v>
       </c>
       <c r="K109" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4503,6 +4832,9 @@
         <v>0</v>
       </c>
       <c r="K110" t="n">
+        <v>0</v>
+      </c>
+      <c r="L110" t="n">
         <v>27</v>
       </c>
     </row>
@@ -4540,6 +4872,9 @@
         <v>0</v>
       </c>
       <c r="K111" t="n">
+        <v>0</v>
+      </c>
+      <c r="L111" t="n">
         <v>19</v>
       </c>
     </row>
@@ -4577,6 +4912,9 @@
         <v>0</v>
       </c>
       <c r="K112" t="n">
+        <v>0</v>
+      </c>
+      <c r="L112" t="n">
         <v>34</v>
       </c>
     </row>
@@ -4614,6 +4952,9 @@
         <v>0</v>
       </c>
       <c r="K113" t="n">
+        <v>0</v>
+      </c>
+      <c r="L113" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4651,6 +4992,9 @@
         <v>0</v>
       </c>
       <c r="K114" t="n">
+        <v>0</v>
+      </c>
+      <c r="L114" t="n">
         <v>40</v>
       </c>
     </row>
@@ -4688,6 +5032,9 @@
         <v>0</v>
       </c>
       <c r="K115" t="n">
+        <v>0</v>
+      </c>
+      <c r="L115" t="n">
         <v>46</v>
       </c>
     </row>
@@ -4725,6 +5072,9 @@
         <v>0</v>
       </c>
       <c r="K116" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" t="n">
         <v>33</v>
       </c>
     </row>
@@ -4762,6 +5112,9 @@
         <v>0</v>
       </c>
       <c r="K117" t="n">
+        <v>0</v>
+      </c>
+      <c r="L117" t="n">
         <v>26</v>
       </c>
     </row>
@@ -4799,6 +5152,9 @@
         <v>0</v>
       </c>
       <c r="K118" t="n">
+        <v>0</v>
+      </c>
+      <c r="L118" t="n">
         <v>31</v>
       </c>
     </row>
@@ -4836,6 +5192,9 @@
         <v>0</v>
       </c>
       <c r="K119" t="n">
+        <v>0</v>
+      </c>
+      <c r="L119" t="n">
         <v>142</v>
       </c>
     </row>
@@ -4873,6 +5232,9 @@
         <v>0</v>
       </c>
       <c r="K120" t="n">
+        <v>0</v>
+      </c>
+      <c r="L120" t="n">
         <v>41</v>
       </c>
     </row>
@@ -4910,6 +5272,9 @@
         <v>0</v>
       </c>
       <c r="K121" t="n">
+        <v>0</v>
+      </c>
+      <c r="L121" t="n">
         <v>34</v>
       </c>
     </row>
@@ -4947,6 +5312,9 @@
         <v>0</v>
       </c>
       <c r="K122" t="n">
+        <v>0</v>
+      </c>
+      <c r="L122" t="n">
         <v>24</v>
       </c>
     </row>
@@ -4984,6 +5352,9 @@
         <v>0</v>
       </c>
       <c r="K123" t="n">
+        <v>0</v>
+      </c>
+      <c r="L123" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5021,6 +5392,9 @@
         <v>0</v>
       </c>
       <c r="K124" t="n">
+        <v>0</v>
+      </c>
+      <c r="L124" t="n">
         <v>98</v>
       </c>
     </row>
@@ -5058,6 +5432,9 @@
         <v>0</v>
       </c>
       <c r="K125" t="n">
+        <v>0</v>
+      </c>
+      <c r="L125" t="n">
         <v>12</v>
       </c>
     </row>
@@ -5095,6 +5472,9 @@
         <v>0</v>
       </c>
       <c r="K126" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" t="n">
         <v>29</v>
       </c>
     </row>
@@ -5132,6 +5512,9 @@
         <v>0</v>
       </c>
       <c r="K127" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" t="n">
         <v>24</v>
       </c>
     </row>
@@ -5169,6 +5552,9 @@
         <v>0</v>
       </c>
       <c r="K128" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" t="n">
         <v>21</v>
       </c>
     </row>
@@ -5206,6 +5592,9 @@
         <v>0</v>
       </c>
       <c r="K129" t="n">
+        <v>0</v>
+      </c>
+      <c r="L129" t="n">
         <v>33</v>
       </c>
     </row>
@@ -5243,6 +5632,9 @@
         <v>0</v>
       </c>
       <c r="K130" t="n">
+        <v>0</v>
+      </c>
+      <c r="L130" t="n">
         <v>5</v>
       </c>
     </row>
@@ -5280,6 +5672,9 @@
         <v>0</v>
       </c>
       <c r="K131" t="n">
+        <v>0</v>
+      </c>
+      <c r="L131" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5317,6 +5712,9 @@
         <v>0</v>
       </c>
       <c r="K132" t="n">
+        <v>0</v>
+      </c>
+      <c r="L132" t="n">
         <v>81</v>
       </c>
     </row>
@@ -5354,6 +5752,9 @@
         <v>0</v>
       </c>
       <c r="K133" t="n">
+        <v>0</v>
+      </c>
+      <c r="L133" t="n">
         <v>25</v>
       </c>
     </row>
@@ -5391,6 +5792,9 @@
         <v>0</v>
       </c>
       <c r="K134" t="n">
+        <v>0</v>
+      </c>
+      <c r="L134" t="n">
         <v>32</v>
       </c>
     </row>
@@ -5428,6 +5832,9 @@
         <v>0</v>
       </c>
       <c r="K135" t="n">
+        <v>0</v>
+      </c>
+      <c r="L135" t="n">
         <v>60</v>
       </c>
     </row>
@@ -5465,6 +5872,9 @@
         <v>0</v>
       </c>
       <c r="K136" t="n">
+        <v>0</v>
+      </c>
+      <c r="L136" t="n">
         <v>28</v>
       </c>
     </row>
@@ -5502,6 +5912,9 @@
         <v>0</v>
       </c>
       <c r="K137" t="n">
+        <v>0</v>
+      </c>
+      <c r="L137" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5539,6 +5952,9 @@
         <v>0</v>
       </c>
       <c r="K138" t="n">
+        <v>0</v>
+      </c>
+      <c r="L138" t="n">
         <v>34</v>
       </c>
     </row>
@@ -5576,6 +5992,9 @@
         <v>0</v>
       </c>
       <c r="K139" t="n">
+        <v>0</v>
+      </c>
+      <c r="L139" t="n">
         <v>45</v>
       </c>
     </row>
@@ -5613,6 +6032,9 @@
         <v>0</v>
       </c>
       <c r="K140" t="n">
+        <v>0</v>
+      </c>
+      <c r="L140" t="n">
         <v>45</v>
       </c>
     </row>
@@ -5650,6 +6072,9 @@
         <v>0</v>
       </c>
       <c r="K141" t="n">
+        <v>0</v>
+      </c>
+      <c r="L141" t="n">
         <v>35</v>
       </c>
     </row>
@@ -5687,6 +6112,9 @@
         <v>0</v>
       </c>
       <c r="K142" t="n">
+        <v>0</v>
+      </c>
+      <c r="L142" t="n">
         <v>29</v>
       </c>
     </row>
@@ -5724,6 +6152,9 @@
         <v>0</v>
       </c>
       <c r="K143" t="n">
+        <v>0</v>
+      </c>
+      <c r="L143" t="n">
         <v>50</v>
       </c>
     </row>
@@ -5761,6 +6192,9 @@
         <v>0</v>
       </c>
       <c r="K144" t="n">
+        <v>0</v>
+      </c>
+      <c r="L144" t="n">
         <v>47</v>
       </c>
     </row>
@@ -5798,6 +6232,9 @@
         <v>0</v>
       </c>
       <c r="K145" t="n">
+        <v>0</v>
+      </c>
+      <c r="L145" t="n">
         <v>77</v>
       </c>
     </row>
@@ -5835,6 +6272,9 @@
         <v>0</v>
       </c>
       <c r="K146" t="n">
+        <v>0</v>
+      </c>
+      <c r="L146" t="n">
         <v>34</v>
       </c>
     </row>
@@ -5872,6 +6312,9 @@
         <v>0</v>
       </c>
       <c r="K147" t="n">
+        <v>0</v>
+      </c>
+      <c r="L147" t="n">
         <v>81</v>
       </c>
     </row>
@@ -5909,6 +6352,9 @@
         <v>0</v>
       </c>
       <c r="K148" t="n">
+        <v>0</v>
+      </c>
+      <c r="L148" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5946,6 +6392,9 @@
         <v>0</v>
       </c>
       <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" t="n">
         <v>47</v>
       </c>
     </row>
@@ -5983,6 +6432,9 @@
         <v>0</v>
       </c>
       <c r="K150" t="n">
+        <v>0</v>
+      </c>
+      <c r="L150" t="n">
         <v>42</v>
       </c>
     </row>
@@ -6020,6 +6472,9 @@
         <v>0</v>
       </c>
       <c r="K151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" t="n">
         <v>30</v>
       </c>
     </row>
@@ -6057,6 +6512,9 @@
         <v>0</v>
       </c>
       <c r="K152" t="n">
+        <v>0</v>
+      </c>
+      <c r="L152" t="n">
         <v>59</v>
       </c>
     </row>
@@ -6094,6 +6552,9 @@
         <v>0</v>
       </c>
       <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" t="n">
         <v>113</v>
       </c>
     </row>
@@ -6131,6 +6592,9 @@
         <v>0</v>
       </c>
       <c r="K154" t="n">
+        <v>0</v>
+      </c>
+      <c r="L154" t="n">
         <v>44</v>
       </c>
     </row>
@@ -6168,6 +6632,9 @@
         <v>0</v>
       </c>
       <c r="K155" t="n">
+        <v>0</v>
+      </c>
+      <c r="L155" t="n">
         <v>52</v>
       </c>
     </row>
@@ -6205,6 +6672,9 @@
         <v>0</v>
       </c>
       <c r="K156" t="n">
+        <v>0</v>
+      </c>
+      <c r="L156" t="n">
         <v>55</v>
       </c>
     </row>
@@ -6242,6 +6712,9 @@
         <v>0</v>
       </c>
       <c r="K157" t="n">
+        <v>0</v>
+      </c>
+      <c r="L157" t="n">
         <v>42</v>
       </c>
     </row>
@@ -6279,6 +6752,9 @@
         <v>0</v>
       </c>
       <c r="K158" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" t="n">
         <v>37</v>
       </c>
     </row>
@@ -6316,6 +6792,9 @@
         <v>0</v>
       </c>
       <c r="K159" t="n">
+        <v>0</v>
+      </c>
+      <c r="L159" t="n">
         <v>27</v>
       </c>
     </row>
@@ -6353,6 +6832,9 @@
         <v>0</v>
       </c>
       <c r="K160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" t="n">
         <v>39</v>
       </c>
     </row>
@@ -6390,6 +6872,9 @@
         <v>0</v>
       </c>
       <c r="K161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" t="n">
         <v>34</v>
       </c>
     </row>
@@ -6427,6 +6912,9 @@
         <v>0</v>
       </c>
       <c r="K162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L162" t="n">
         <v>32</v>
       </c>
     </row>
@@ -6464,6 +6952,9 @@
         <v>0</v>
       </c>
       <c r="K163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L163" t="n">
         <v>137</v>
       </c>
     </row>
@@ -6501,6 +6992,9 @@
         <v>0</v>
       </c>
       <c r="K164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L164" t="n">
         <v>40</v>
       </c>
     </row>
@@ -6538,6 +7032,9 @@
         <v>0</v>
       </c>
       <c r="K165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" t="n">
         <v>119</v>
       </c>
     </row>
@@ -6575,6 +7072,9 @@
         <v>0</v>
       </c>
       <c r="K166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L166" t="n">
         <v>40</v>
       </c>
     </row>
@@ -6612,6 +7112,9 @@
         <v>0</v>
       </c>
       <c r="K167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L167" t="n">
         <v>70</v>
       </c>
     </row>
@@ -6649,6 +7152,9 @@
         <v>0</v>
       </c>
       <c r="K168" t="n">
+        <v>0</v>
+      </c>
+      <c r="L168" t="n">
         <v>73</v>
       </c>
     </row>
@@ -6686,6 +7192,9 @@
         <v>0</v>
       </c>
       <c r="K169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L169" t="n">
         <v>50</v>
       </c>
     </row>
@@ -6723,6 +7232,9 @@
         <v>0</v>
       </c>
       <c r="K170" t="n">
+        <v>0</v>
+      </c>
+      <c r="L170" t="n">
         <v>71</v>
       </c>
     </row>
@@ -6760,6 +7272,9 @@
         <v>0</v>
       </c>
       <c r="K171" t="n">
+        <v>0</v>
+      </c>
+      <c r="L171" t="n">
         <v>126</v>
       </c>
     </row>
@@ -6797,6 +7312,9 @@
         <v>0</v>
       </c>
       <c r="K172" t="n">
+        <v>0</v>
+      </c>
+      <c r="L172" t="n">
         <v>115</v>
       </c>
     </row>
@@ -6834,6 +7352,9 @@
         <v>0</v>
       </c>
       <c r="K173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L173" t="n">
         <v>38</v>
       </c>
     </row>
@@ -6871,6 +7392,9 @@
         <v>0</v>
       </c>
       <c r="K174" t="n">
+        <v>0</v>
+      </c>
+      <c r="L174" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6908,6 +7432,9 @@
         <v>0</v>
       </c>
       <c r="K175" t="n">
+        <v>0</v>
+      </c>
+      <c r="L175" t="n">
         <v>138</v>
       </c>
     </row>
@@ -6945,6 +7472,9 @@
         <v>0</v>
       </c>
       <c r="K176" t="n">
+        <v>0</v>
+      </c>
+      <c r="L176" t="n">
         <v>129</v>
       </c>
     </row>
@@ -6982,6 +7512,9 @@
         <v>0</v>
       </c>
       <c r="K177" t="n">
+        <v>0</v>
+      </c>
+      <c r="L177" t="n">
         <v>50</v>
       </c>
     </row>
@@ -7019,6 +7552,9 @@
         <v>0</v>
       </c>
       <c r="K178" t="n">
+        <v>0</v>
+      </c>
+      <c r="L178" t="n">
         <v>68</v>
       </c>
     </row>
@@ -7056,6 +7592,9 @@
         <v>0</v>
       </c>
       <c r="K179" t="n">
+        <v>0</v>
+      </c>
+      <c r="L179" t="n">
         <v>33</v>
       </c>
     </row>
@@ -7093,6 +7632,9 @@
         <v>0</v>
       </c>
       <c r="K180" t="n">
+        <v>0</v>
+      </c>
+      <c r="L180" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7130,6 +7672,9 @@
         <v>0</v>
       </c>
       <c r="K181" t="n">
+        <v>0</v>
+      </c>
+      <c r="L181" t="n">
         <v>133</v>
       </c>
     </row>
@@ -7167,6 +7712,9 @@
         <v>0</v>
       </c>
       <c r="K182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L182" t="n">
         <v>125</v>
       </c>
     </row>
@@ -7204,6 +7752,9 @@
         <v>0</v>
       </c>
       <c r="K183" t="n">
+        <v>0</v>
+      </c>
+      <c r="L183" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7241,6 +7792,9 @@
         <v>0</v>
       </c>
       <c r="K184" t="n">
+        <v>0</v>
+      </c>
+      <c r="L184" t="n">
         <v>84</v>
       </c>
     </row>
@@ -7278,6 +7832,9 @@
         <v>0</v>
       </c>
       <c r="K185" t="n">
+        <v>0</v>
+      </c>
+      <c r="L185" t="n">
         <v>58</v>
       </c>
     </row>
@@ -7315,6 +7872,9 @@
         <v>0</v>
       </c>
       <c r="K186" t="n">
+        <v>0</v>
+      </c>
+      <c r="L186" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7352,6 +7912,9 @@
         <v>0</v>
       </c>
       <c r="K187" t="n">
+        <v>0</v>
+      </c>
+      <c r="L187" t="n">
         <v>104</v>
       </c>
     </row>
@@ -7389,6 +7952,9 @@
         <v>0</v>
       </c>
       <c r="K188" t="n">
+        <v>0</v>
+      </c>
+      <c r="L188" t="n">
         <v>63</v>
       </c>
     </row>
@@ -7426,6 +7992,9 @@
         <v>0</v>
       </c>
       <c r="K189" t="n">
+        <v>0</v>
+      </c>
+      <c r="L189" t="n">
         <v>62</v>
       </c>
     </row>
@@ -7463,6 +8032,9 @@
         <v>0</v>
       </c>
       <c r="K190" t="n">
+        <v>0</v>
+      </c>
+      <c r="L190" t="n">
         <v>58</v>
       </c>
     </row>
@@ -7500,6 +8072,9 @@
         <v>0</v>
       </c>
       <c r="K191" t="n">
+        <v>0</v>
+      </c>
+      <c r="L191" t="n">
         <v>45</v>
       </c>
     </row>
@@ -7537,6 +8112,9 @@
         <v>0</v>
       </c>
       <c r="K192" t="n">
+        <v>0</v>
+      </c>
+      <c r="L192" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7574,6 +8152,9 @@
         <v>0</v>
       </c>
       <c r="K193" t="n">
+        <v>0</v>
+      </c>
+      <c r="L193" t="n">
         <v>182</v>
       </c>
     </row>
@@ -7611,6 +8192,9 @@
         <v>0</v>
       </c>
       <c r="K194" t="n">
+        <v>0</v>
+      </c>
+      <c r="L194" t="n">
         <v>4</v>
       </c>
     </row>
@@ -7648,6 +8232,9 @@
         <v>0</v>
       </c>
       <c r="K195" t="n">
+        <v>0</v>
+      </c>
+      <c r="L195" t="n">
         <v>105</v>
       </c>
     </row>
@@ -7685,6 +8272,9 @@
         <v>0</v>
       </c>
       <c r="K196" t="n">
+        <v>0</v>
+      </c>
+      <c r="L196" t="n">
         <v>102</v>
       </c>
     </row>
@@ -7722,6 +8312,9 @@
         <v>0</v>
       </c>
       <c r="K197" t="n">
+        <v>0</v>
+      </c>
+      <c r="L197" t="n">
         <v>28</v>
       </c>
     </row>
@@ -7759,6 +8352,9 @@
         <v>0</v>
       </c>
       <c r="K198" t="n">
+        <v>0</v>
+      </c>
+      <c r="L198" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7796,6 +8392,9 @@
         <v>0</v>
       </c>
       <c r="K199" t="n">
+        <v>0</v>
+      </c>
+      <c r="L199" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7833,6 +8432,9 @@
         <v>0</v>
       </c>
       <c r="K200" t="n">
+        <v>0</v>
+      </c>
+      <c r="L200" t="n">
         <v>15</v>
       </c>
     </row>
@@ -7870,6 +8472,9 @@
         <v>0</v>
       </c>
       <c r="K201" t="n">
+        <v>0</v>
+      </c>
+      <c r="L201" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7907,6 +8512,9 @@
         <v>0</v>
       </c>
       <c r="K202" t="n">
+        <v>0</v>
+      </c>
+      <c r="L202" t="n">
         <v>24</v>
       </c>
     </row>
@@ -7944,6 +8552,9 @@
         <v>0</v>
       </c>
       <c r="K203" t="n">
+        <v>0</v>
+      </c>
+      <c r="L203" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7981,6 +8592,9 @@
         <v>0</v>
       </c>
       <c r="K204" t="n">
+        <v>0</v>
+      </c>
+      <c r="L204" t="n">
         <v>17</v>
       </c>
     </row>
@@ -8018,6 +8632,9 @@
         <v>0</v>
       </c>
       <c r="K205" t="n">
+        <v>0</v>
+      </c>
+      <c r="L205" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8055,6 +8672,9 @@
         <v>0</v>
       </c>
       <c r="K206" t="n">
+        <v>0</v>
+      </c>
+      <c r="L206" t="n">
         <v>22</v>
       </c>
     </row>
@@ -8092,6 +8712,9 @@
         <v>0</v>
       </c>
       <c r="K207" t="n">
+        <v>0</v>
+      </c>
+      <c r="L207" t="n">
         <v>27</v>
       </c>
     </row>
@@ -8129,6 +8752,9 @@
         <v>0</v>
       </c>
       <c r="K208" t="n">
+        <v>0</v>
+      </c>
+      <c r="L208" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8166,6 +8792,9 @@
         <v>0</v>
       </c>
       <c r="K209" t="n">
+        <v>0</v>
+      </c>
+      <c r="L209" t="n">
         <v>53</v>
       </c>
     </row>
@@ -8203,6 +8832,9 @@
         <v>0</v>
       </c>
       <c r="K210" t="n">
+        <v>0</v>
+      </c>
+      <c r="L210" t="n">
         <v>33</v>
       </c>
     </row>
@@ -8240,6 +8872,9 @@
         <v>0</v>
       </c>
       <c r="K211" t="n">
+        <v>0</v>
+      </c>
+      <c r="L211" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8277,6 +8912,9 @@
         <v>0</v>
       </c>
       <c r="K212" t="n">
+        <v>0</v>
+      </c>
+      <c r="L212" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8314,6 +8952,9 @@
         <v>0</v>
       </c>
       <c r="K213" t="n">
+        <v>0</v>
+      </c>
+      <c r="L213" t="n">
         <v>59</v>
       </c>
     </row>
@@ -8351,6 +8992,9 @@
         <v>0</v>
       </c>
       <c r="K214" t="n">
+        <v>0</v>
+      </c>
+      <c r="L214" t="n">
         <v>29</v>
       </c>
     </row>
@@ -8388,6 +9032,9 @@
         <v>0</v>
       </c>
       <c r="K215" t="n">
+        <v>0</v>
+      </c>
+      <c r="L215" t="n">
         <v>25</v>
       </c>
     </row>
@@ -8425,6 +9072,9 @@
         <v>0</v>
       </c>
       <c r="K216" t="n">
+        <v>0</v>
+      </c>
+      <c r="L216" t="n">
         <v>26</v>
       </c>
     </row>
@@ -8462,6 +9112,9 @@
         <v>0</v>
       </c>
       <c r="K217" t="n">
+        <v>0</v>
+      </c>
+      <c r="L217" t="n">
         <v>23</v>
       </c>
     </row>
@@ -8499,6 +9152,9 @@
         <v>0</v>
       </c>
       <c r="K218" t="n">
+        <v>0</v>
+      </c>
+      <c r="L218" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8536,6 +9192,9 @@
         <v>0</v>
       </c>
       <c r="K219" t="n">
+        <v>0</v>
+      </c>
+      <c r="L219" t="n">
         <v>48</v>
       </c>
     </row>
@@ -8573,6 +9232,9 @@
         <v>0</v>
       </c>
       <c r="K220" t="n">
+        <v>0</v>
+      </c>
+      <c r="L220" t="n">
         <v>39</v>
       </c>
     </row>
@@ -8610,6 +9272,9 @@
         <v>0</v>
       </c>
       <c r="K221" t="n">
+        <v>0</v>
+      </c>
+      <c r="L221" t="n">
         <v>41</v>
       </c>
     </row>
@@ -8647,6 +9312,9 @@
         <v>0</v>
       </c>
       <c r="K222" t="n">
+        <v>0</v>
+      </c>
+      <c r="L222" t="n">
         <v>65</v>
       </c>
     </row>
@@ -8684,6 +9352,9 @@
         <v>0</v>
       </c>
       <c r="K223" t="n">
+        <v>0</v>
+      </c>
+      <c r="L223" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8721,6 +9392,9 @@
         <v>0</v>
       </c>
       <c r="K224" t="n">
+        <v>0</v>
+      </c>
+      <c r="L224" t="n">
         <v>89</v>
       </c>
     </row>
@@ -8758,6 +9432,9 @@
         <v>0</v>
       </c>
       <c r="K225" t="n">
+        <v>0</v>
+      </c>
+      <c r="L225" t="n">
         <v>58</v>
       </c>
     </row>
@@ -8795,6 +9472,9 @@
         <v>0</v>
       </c>
       <c r="K226" t="n">
+        <v>0</v>
+      </c>
+      <c r="L226" t="n">
         <v>73</v>
       </c>
     </row>
@@ -8832,6 +9512,9 @@
         <v>0</v>
       </c>
       <c r="K227" t="n">
+        <v>0</v>
+      </c>
+      <c r="L227" t="n">
         <v>199</v>
       </c>
     </row>
@@ -8869,6 +9552,9 @@
         <v>0</v>
       </c>
       <c r="K228" t="n">
+        <v>0</v>
+      </c>
+      <c r="L228" t="n">
         <v>94</v>
       </c>
     </row>
@@ -8906,6 +9592,9 @@
         <v>0</v>
       </c>
       <c r="K229" t="n">
+        <v>0</v>
+      </c>
+      <c r="L229" t="n">
         <v>139</v>
       </c>
     </row>
@@ -8943,6 +9632,9 @@
         <v>0</v>
       </c>
       <c r="K230" t="n">
+        <v>0</v>
+      </c>
+      <c r="L230" t="n">
         <v>2</v>
       </c>
     </row>
@@ -8980,6 +9672,9 @@
         <v>0</v>
       </c>
       <c r="K231" t="n">
+        <v>0</v>
+      </c>
+      <c r="L231" t="n">
         <v>168</v>
       </c>
     </row>
@@ -9017,6 +9712,9 @@
         <v>0</v>
       </c>
       <c r="K232" t="n">
+        <v>0</v>
+      </c>
+      <c r="L232" t="n">
         <v>71</v>
       </c>
     </row>
@@ -9054,6 +9752,9 @@
         <v>0</v>
       </c>
       <c r="K233" t="n">
+        <v>0</v>
+      </c>
+      <c r="L233" t="n">
         <v>77</v>
       </c>
     </row>
@@ -9091,6 +9792,9 @@
         <v>0</v>
       </c>
       <c r="K234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L234" t="n">
         <v>46</v>
       </c>
     </row>
@@ -9128,6 +9832,9 @@
         <v>0</v>
       </c>
       <c r="K235" t="n">
+        <v>0</v>
+      </c>
+      <c r="L235" t="n">
         <v>42</v>
       </c>
     </row>
@@ -9165,6 +9872,9 @@
         <v>0</v>
       </c>
       <c r="K236" t="n">
+        <v>0</v>
+      </c>
+      <c r="L236" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9202,6 +9912,9 @@
         <v>0</v>
       </c>
       <c r="K237" t="n">
+        <v>0</v>
+      </c>
+      <c r="L237" t="n">
         <v>204</v>
       </c>
     </row>
@@ -9239,6 +9952,9 @@
         <v>0</v>
       </c>
       <c r="K238" t="n">
+        <v>0</v>
+      </c>
+      <c r="L238" t="n">
         <v>50</v>
       </c>
     </row>
@@ -9276,6 +9992,9 @@
         <v>0</v>
       </c>
       <c r="K239" t="n">
+        <v>0</v>
+      </c>
+      <c r="L239" t="n">
         <v>32</v>
       </c>
     </row>
@@ -9313,6 +10032,9 @@
         <v>0</v>
       </c>
       <c r="K240" t="n">
+        <v>0</v>
+      </c>
+      <c r="L240" t="n">
         <v>61</v>
       </c>
     </row>
@@ -9350,6 +10072,9 @@
         <v>0</v>
       </c>
       <c r="K241" t="n">
+        <v>0</v>
+      </c>
+      <c r="L241" t="n">
         <v>43</v>
       </c>
     </row>
@@ -9387,6 +10112,9 @@
         <v>0</v>
       </c>
       <c r="K242" t="n">
+        <v>0</v>
+      </c>
+      <c r="L242" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9424,6 +10152,9 @@
         <v>0</v>
       </c>
       <c r="K243" t="n">
+        <v>0</v>
+      </c>
+      <c r="L243" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9461,6 +10192,9 @@
         <v>0</v>
       </c>
       <c r="K244" t="n">
+        <v>0</v>
+      </c>
+      <c r="L244" t="n">
         <v>2</v>
       </c>
     </row>
@@ -9498,6 +10232,9 @@
         <v>0</v>
       </c>
       <c r="K245" t="n">
+        <v>0</v>
+      </c>
+      <c r="L245" t="n">
         <v>60</v>
       </c>
     </row>
@@ -9535,6 +10272,9 @@
         <v>0</v>
       </c>
       <c r="K246" t="n">
+        <v>0</v>
+      </c>
+      <c r="L246" t="n">
         <v>152</v>
       </c>
     </row>
@@ -9572,6 +10312,9 @@
         <v>0</v>
       </c>
       <c r="K247" t="n">
+        <v>0</v>
+      </c>
+      <c r="L247" t="n">
         <v>236</v>
       </c>
     </row>
@@ -9609,6 +10352,9 @@
         <v>0</v>
       </c>
       <c r="K248" t="n">
+        <v>0</v>
+      </c>
+      <c r="L248" t="n">
         <v>72</v>
       </c>
     </row>
@@ -9646,6 +10392,9 @@
         <v>0</v>
       </c>
       <c r="K249" t="n">
+        <v>0</v>
+      </c>
+      <c r="L249" t="n">
         <v>6</v>
       </c>
     </row>
@@ -9683,6 +10432,9 @@
         <v>0</v>
       </c>
       <c r="K250" t="n">
+        <v>0</v>
+      </c>
+      <c r="L250" t="n">
         <v>6</v>
       </c>
     </row>
@@ -9720,6 +10472,9 @@
         <v>0</v>
       </c>
       <c r="K251" t="n">
+        <v>0</v>
+      </c>
+      <c r="L251" t="n">
         <v>296</v>
       </c>
     </row>
@@ -9757,6 +10512,9 @@
         <v>0</v>
       </c>
       <c r="K252" t="n">
+        <v>0</v>
+      </c>
+      <c r="L252" t="n">
         <v>1172</v>
       </c>
     </row>
@@ -9794,6 +10552,9 @@
         <v>0</v>
       </c>
       <c r="K253" t="n">
+        <v>0</v>
+      </c>
+      <c r="L253" t="n">
         <v>161</v>
       </c>
     </row>
@@ -9831,6 +10592,9 @@
         <v>0</v>
       </c>
       <c r="K254" t="n">
+        <v>0</v>
+      </c>
+      <c r="L254" t="n">
         <v>173</v>
       </c>
     </row>
@@ -9868,6 +10632,9 @@
         <v>0</v>
       </c>
       <c r="K255" t="n">
+        <v>0</v>
+      </c>
+      <c r="L255" t="n">
         <v>192</v>
       </c>
     </row>
@@ -9905,6 +10672,9 @@
         <v>0</v>
       </c>
       <c r="K256" t="n">
+        <v>0</v>
+      </c>
+      <c r="L256" t="n">
         <v>269</v>
       </c>
     </row>
@@ -9942,6 +10712,9 @@
         <v>0</v>
       </c>
       <c r="K257" t="n">
+        <v>0</v>
+      </c>
+      <c r="L257" t="n">
         <v>61</v>
       </c>
     </row>
@@ -9979,6 +10752,9 @@
         <v>0</v>
       </c>
       <c r="K258" t="n">
+        <v>0</v>
+      </c>
+      <c r="L258" t="n">
         <v>135</v>
       </c>
     </row>
@@ -10016,6 +10792,9 @@
         <v>0</v>
       </c>
       <c r="K259" t="n">
+        <v>0</v>
+      </c>
+      <c r="L259" t="n">
         <v>67</v>
       </c>
     </row>
@@ -10053,6 +10832,9 @@
         <v>0</v>
       </c>
       <c r="K260" t="n">
+        <v>0</v>
+      </c>
+      <c r="L260" t="n">
         <v>12</v>
       </c>
     </row>
@@ -10090,6 +10872,9 @@
         <v>0</v>
       </c>
       <c r="K261" t="n">
+        <v>0</v>
+      </c>
+      <c r="L261" t="n">
         <v>64</v>
       </c>
     </row>
@@ -10127,6 +10912,9 @@
         <v>0</v>
       </c>
       <c r="K262" t="n">
+        <v>0</v>
+      </c>
+      <c r="L262" t="n">
         <v>49</v>
       </c>
     </row>
@@ -10164,6 +10952,9 @@
         <v>0</v>
       </c>
       <c r="K263" t="n">
+        <v>0</v>
+      </c>
+      <c r="L263" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10201,6 +10992,9 @@
         <v>0</v>
       </c>
       <c r="K264" t="n">
+        <v>0</v>
+      </c>
+      <c r="L264" t="n">
         <v>30</v>
       </c>
     </row>
@@ -10238,6 +11032,9 @@
         <v>0</v>
       </c>
       <c r="K265" t="n">
+        <v>0</v>
+      </c>
+      <c r="L265" t="n">
         <v>233</v>
       </c>
     </row>
@@ -10275,6 +11072,9 @@
         <v>0</v>
       </c>
       <c r="K266" t="n">
+        <v>0</v>
+      </c>
+      <c r="L266" t="n">
         <v>274</v>
       </c>
     </row>
@@ -10312,6 +11112,9 @@
         <v>0</v>
       </c>
       <c r="K267" t="n">
+        <v>0</v>
+      </c>
+      <c r="L267" t="n">
         <v>85</v>
       </c>
     </row>
@@ -10349,6 +11152,9 @@
         <v>3</v>
       </c>
       <c r="K268" t="n">
+        <v>0</v>
+      </c>
+      <c r="L268" t="n">
         <v>103</v>
       </c>
     </row>
@@ -10386,6 +11192,9 @@
         <v>0</v>
       </c>
       <c r="K269" t="n">
+        <v>0</v>
+      </c>
+      <c r="L269" t="n">
         <v>93</v>
       </c>
     </row>
@@ -10423,6 +11232,9 @@
         <v>2</v>
       </c>
       <c r="K270" t="n">
+        <v>0</v>
+      </c>
+      <c r="L270" t="n">
         <v>5</v>
       </c>
     </row>
@@ -10460,6 +11272,9 @@
         <v>1</v>
       </c>
       <c r="K271" t="n">
+        <v>0</v>
+      </c>
+      <c r="L271" t="n">
         <v>146</v>
       </c>
     </row>
@@ -10470,7 +11285,7 @@
         </is>
       </c>
       <c r="B272" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C272" t="n">
         <v>0</v>
@@ -10497,7 +11312,10 @@
         <v>0</v>
       </c>
       <c r="K272" t="n">
-        <v>155</v>
+        <v>0</v>
+      </c>
+      <c r="L272" t="n">
+        <v>156</v>
       </c>
     </row>
     <row r="273">
@@ -10534,6 +11352,9 @@
         <v>2</v>
       </c>
       <c r="K273" t="n">
+        <v>0</v>
+      </c>
+      <c r="L273" t="n">
         <v>104</v>
       </c>
     </row>
@@ -10544,7 +11365,7 @@
         </is>
       </c>
       <c r="B274" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C274" t="n">
         <v>0</v>
@@ -10571,7 +11392,10 @@
         <v>1</v>
       </c>
       <c r="K274" t="n">
-        <v>104</v>
+        <v>0</v>
+      </c>
+      <c r="L274" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="275">
@@ -10608,6 +11432,9 @@
         <v>1</v>
       </c>
       <c r="K275" t="n">
+        <v>0</v>
+      </c>
+      <c r="L275" t="n">
         <v>101</v>
       </c>
     </row>
@@ -10645,6 +11472,9 @@
         <v>5</v>
       </c>
       <c r="K276" t="n">
+        <v>0</v>
+      </c>
+      <c r="L276" t="n">
         <v>122</v>
       </c>
     </row>
@@ -10682,6 +11512,9 @@
         <v>1</v>
       </c>
       <c r="K277" t="n">
+        <v>0</v>
+      </c>
+      <c r="L277" t="n">
         <v>298</v>
       </c>
     </row>
@@ -10719,6 +11552,9 @@
         <v>3</v>
       </c>
       <c r="K278" t="n">
+        <v>0</v>
+      </c>
+      <c r="L278" t="n">
         <v>30</v>
       </c>
     </row>
@@ -10756,6 +11592,9 @@
         <v>2</v>
       </c>
       <c r="K279" t="n">
+        <v>0</v>
+      </c>
+      <c r="L279" t="n">
         <v>38</v>
       </c>
     </row>
@@ -10793,6 +11632,9 @@
         <v>3</v>
       </c>
       <c r="K280" t="n">
+        <v>0</v>
+      </c>
+      <c r="L280" t="n">
         <v>110</v>
       </c>
     </row>
@@ -10803,7 +11645,7 @@
         </is>
       </c>
       <c r="B281" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C281" t="n">
         <v>0</v>
@@ -10830,7 +11672,10 @@
         <v>2</v>
       </c>
       <c r="K281" t="n">
-        <v>313</v>
+        <v>0</v>
+      </c>
+      <c r="L281" t="n">
+        <v>314</v>
       </c>
     </row>
     <row r="282">
@@ -10840,7 +11685,7 @@
         </is>
       </c>
       <c r="B282" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C282" t="n">
         <v>0</v>
@@ -10867,7 +11712,10 @@
         <v>3</v>
       </c>
       <c r="K282" t="n">
-        <v>129</v>
+        <v>0</v>
+      </c>
+      <c r="L282" t="n">
+        <v>131</v>
       </c>
     </row>
     <row r="283">
@@ -10904,6 +11752,9 @@
         <v>1</v>
       </c>
       <c r="K283" t="n">
+        <v>0</v>
+      </c>
+      <c r="L283" t="n">
         <v>26</v>
       </c>
     </row>
@@ -10941,6 +11792,9 @@
         <v>0</v>
       </c>
       <c r="K284" t="n">
+        <v>0</v>
+      </c>
+      <c r="L284" t="n">
         <v>25</v>
       </c>
     </row>
@@ -10978,6 +11832,9 @@
         <v>0</v>
       </c>
       <c r="K285" t="n">
+        <v>0</v>
+      </c>
+      <c r="L285" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11015,6 +11872,9 @@
         <v>0</v>
       </c>
       <c r="K286" t="n">
+        <v>0</v>
+      </c>
+      <c r="L286" t="n">
         <v>147</v>
       </c>
     </row>
@@ -11052,6 +11912,9 @@
         <v>0</v>
       </c>
       <c r="K287" t="n">
+        <v>0</v>
+      </c>
+      <c r="L287" t="n">
         <v>130</v>
       </c>
     </row>
@@ -11089,6 +11952,9 @@
         <v>0</v>
       </c>
       <c r="K288" t="n">
+        <v>0</v>
+      </c>
+      <c r="L288" t="n">
         <v>52</v>
       </c>
     </row>
@@ -11126,6 +11992,9 @@
         <v>0</v>
       </c>
       <c r="K289" t="n">
+        <v>0</v>
+      </c>
+      <c r="L289" t="n">
         <v>21</v>
       </c>
     </row>
@@ -11163,6 +12032,9 @@
         <v>0</v>
       </c>
       <c r="K290" t="n">
+        <v>0</v>
+      </c>
+      <c r="L290" t="n">
         <v>46</v>
       </c>
     </row>
@@ -11200,6 +12072,9 @@
         <v>0</v>
       </c>
       <c r="K291" t="n">
+        <v>0</v>
+      </c>
+      <c r="L291" t="n">
         <v>19</v>
       </c>
     </row>
@@ -11237,6 +12112,9 @@
         <v>0</v>
       </c>
       <c r="K292" t="n">
+        <v>0</v>
+      </c>
+      <c r="L292" t="n">
         <v>26</v>
       </c>
     </row>
@@ -11274,6 +12152,9 @@
         <v>0</v>
       </c>
       <c r="K293" t="n">
+        <v>0</v>
+      </c>
+      <c r="L293" t="n">
         <v>28</v>
       </c>
     </row>
@@ -11311,6 +12192,9 @@
         <v>0</v>
       </c>
       <c r="K294" t="n">
+        <v>0</v>
+      </c>
+      <c r="L294" t="n">
         <v>227</v>
       </c>
     </row>
@@ -11348,6 +12232,9 @@
         <v>0</v>
       </c>
       <c r="K295" t="n">
+        <v>0</v>
+      </c>
+      <c r="L295" t="n">
         <v>49</v>
       </c>
     </row>
@@ -11385,6 +12272,9 @@
         <v>0</v>
       </c>
       <c r="K296" t="n">
+        <v>0</v>
+      </c>
+      <c r="L296" t="n">
         <v>74</v>
       </c>
     </row>
@@ -11422,6 +12312,9 @@
         <v>0</v>
       </c>
       <c r="K297" t="n">
+        <v>0</v>
+      </c>
+      <c r="L297" t="n">
         <v>104</v>
       </c>
     </row>
@@ -11459,6 +12352,9 @@
         <v>0</v>
       </c>
       <c r="K298" t="n">
+        <v>0</v>
+      </c>
+      <c r="L298" t="n">
         <v>14</v>
       </c>
     </row>
@@ -11496,6 +12392,9 @@
         <v>0</v>
       </c>
       <c r="K299" t="n">
+        <v>0</v>
+      </c>
+      <c r="L299" t="n">
         <v>15</v>
       </c>
     </row>
@@ -11533,6 +12432,9 @@
         <v>0</v>
       </c>
       <c r="K300" t="n">
+        <v>0</v>
+      </c>
+      <c r="L300" t="n">
         <v>100</v>
       </c>
     </row>
@@ -11570,6 +12472,9 @@
         <v>0</v>
       </c>
       <c r="K301" t="n">
+        <v>0</v>
+      </c>
+      <c r="L301" t="n">
         <v>126</v>
       </c>
     </row>
@@ -11607,6 +12512,9 @@
         <v>0</v>
       </c>
       <c r="K302" t="n">
+        <v>0</v>
+      </c>
+      <c r="L302" t="n">
         <v>37</v>
       </c>
     </row>
@@ -11644,6 +12552,9 @@
         <v>0</v>
       </c>
       <c r="K303" t="n">
+        <v>0</v>
+      </c>
+      <c r="L303" t="n">
         <v>283</v>
       </c>
     </row>
@@ -11681,6 +12592,9 @@
         <v>0</v>
       </c>
       <c r="K304" t="n">
+        <v>0</v>
+      </c>
+      <c r="L304" t="n">
         <v>393</v>
       </c>
     </row>
@@ -11718,6 +12632,9 @@
         <v>0</v>
       </c>
       <c r="K305" t="n">
+        <v>0</v>
+      </c>
+      <c r="L305" t="n">
         <v>373</v>
       </c>
     </row>
@@ -11755,6 +12672,9 @@
         <v>0</v>
       </c>
       <c r="K306" t="n">
+        <v>0</v>
+      </c>
+      <c r="L306" t="n">
         <v>204</v>
       </c>
     </row>
@@ -11792,6 +12712,9 @@
         <v>0</v>
       </c>
       <c r="K307" t="n">
+        <v>0</v>
+      </c>
+      <c r="L307" t="n">
         <v>95</v>
       </c>
     </row>
@@ -11829,6 +12752,9 @@
         <v>0</v>
       </c>
       <c r="K308" t="n">
+        <v>0</v>
+      </c>
+      <c r="L308" t="n">
         <v>110</v>
       </c>
     </row>
@@ -11866,6 +12792,9 @@
         <v>0</v>
       </c>
       <c r="K309" t="n">
+        <v>0</v>
+      </c>
+      <c r="L309" t="n">
         <v>109</v>
       </c>
     </row>
@@ -11903,6 +12832,9 @@
         <v>0</v>
       </c>
       <c r="K310" t="n">
+        <v>0</v>
+      </c>
+      <c r="L310" t="n">
         <v>31</v>
       </c>
     </row>
@@ -11940,6 +12872,9 @@
         <v>0</v>
       </c>
       <c r="K311" t="n">
+        <v>0</v>
+      </c>
+      <c r="L311" t="n">
         <v>34</v>
       </c>
     </row>
@@ -11977,6 +12912,9 @@
         <v>0</v>
       </c>
       <c r="K312" t="n">
+        <v>0</v>
+      </c>
+      <c r="L312" t="n">
         <v>46</v>
       </c>
     </row>
@@ -12014,6 +12952,9 @@
         <v>0</v>
       </c>
       <c r="K313" t="n">
+        <v>0</v>
+      </c>
+      <c r="L313" t="n">
         <v>23</v>
       </c>
     </row>
@@ -12051,6 +12992,9 @@
         <v>0</v>
       </c>
       <c r="K314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L314" t="n">
         <v>15</v>
       </c>
     </row>
@@ -12088,6 +13032,9 @@
         <v>0</v>
       </c>
       <c r="K315" t="n">
+        <v>0</v>
+      </c>
+      <c r="L315" t="n">
         <v>32</v>
       </c>
     </row>
@@ -12125,6 +13072,9 @@
         <v>0</v>
       </c>
       <c r="K316" t="n">
+        <v>0</v>
+      </c>
+      <c r="L316" t="n">
         <v>31</v>
       </c>
     </row>
@@ -12162,6 +13112,9 @@
         <v>0</v>
       </c>
       <c r="K317" t="n">
+        <v>0</v>
+      </c>
+      <c r="L317" t="n">
         <v>46</v>
       </c>
     </row>
@@ -12199,6 +13152,9 @@
         <v>0</v>
       </c>
       <c r="K318" t="n">
+        <v>0</v>
+      </c>
+      <c r="L318" t="n">
         <v>22</v>
       </c>
     </row>
@@ -12236,6 +13192,9 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
+        <v>0</v>
+      </c>
+      <c r="L319" t="n">
         <v>23</v>
       </c>
     </row>
@@ -12273,6 +13232,9 @@
         <v>0</v>
       </c>
       <c r="K320" t="n">
+        <v>0</v>
+      </c>
+      <c r="L320" t="n">
         <v>19</v>
       </c>
     </row>
@@ -12283,10 +13245,10 @@
         </is>
       </c>
       <c r="B321" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="C321" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="D321" t="n">
         <v>0</v>
@@ -12295,13 +13257,13 @@
         <v>0</v>
       </c>
       <c r="F321" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G321" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H321" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I321" t="n">
         <v>0</v>
@@ -12310,7 +13272,10 @@
         <v>0</v>
       </c>
       <c r="K321" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="L321" t="n">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-08 13:01
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L336"/>
+  <dimension ref="A1:L338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13878,6 +13878,86 @@
         <v>1</v>
       </c>
     </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>2</v>
+      </c>
+      <c r="C337" t="n">
+        <v>4</v>
+      </c>
+      <c r="D337" t="n">
+        <v>0</v>
+      </c>
+      <c r="E337" t="n">
+        <v>0</v>
+      </c>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" t="n">
+        <v>1</v>
+      </c>
+      <c r="H337" t="n">
+        <v>0</v>
+      </c>
+      <c r="I337" t="n">
+        <v>0</v>
+      </c>
+      <c r="J337" t="n">
+        <v>0</v>
+      </c>
+      <c r="K337" t="n">
+        <v>0</v>
+      </c>
+      <c r="L337" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B338" t="n">
+        <v>1</v>
+      </c>
+      <c r="C338" t="n">
+        <v>2</v>
+      </c>
+      <c r="D338" t="n">
+        <v>0</v>
+      </c>
+      <c r="E338" t="n">
+        <v>0</v>
+      </c>
+      <c r="F338" t="n">
+        <v>0</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0</v>
+      </c>
+      <c r="H338" t="n">
+        <v>0</v>
+      </c>
+      <c r="I338" t="n">
+        <v>0</v>
+      </c>
+      <c r="J338" t="n">
+        <v>0</v>
+      </c>
+      <c r="K338" t="n">
+        <v>0</v>
+      </c>
+      <c r="L338" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-10 11:00
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L338"/>
+  <dimension ref="A1:L339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13958,6 +13958,46 @@
         <v>54</v>
       </c>
     </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>5</v>
+      </c>
+      <c r="C339" t="n">
+        <v>16</v>
+      </c>
+      <c r="D339" t="n">
+        <v>0</v>
+      </c>
+      <c r="E339" t="n">
+        <v>0</v>
+      </c>
+      <c r="F339" t="n">
+        <v>0</v>
+      </c>
+      <c r="G339" t="n">
+        <v>1</v>
+      </c>
+      <c r="H339" t="n">
+        <v>0</v>
+      </c>
+      <c r="I339" t="n">
+        <v>0</v>
+      </c>
+      <c r="J339" t="n">
+        <v>0</v>
+      </c>
+      <c r="K339" t="n">
+        <v>0</v>
+      </c>
+      <c r="L339" t="n">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-11 13:02
</commit_message>
<xml_diff>
--- a/daily_product_units.xlsx
+++ b/daily_product_units.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L339"/>
+  <dimension ref="A1:L340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13998,6 +13998,46 @@
         <v>22</v>
       </c>
     </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B340" t="n">
+        <v>3</v>
+      </c>
+      <c r="C340" t="n">
+        <v>10</v>
+      </c>
+      <c r="D340" t="n">
+        <v>0</v>
+      </c>
+      <c r="E340" t="n">
+        <v>0</v>
+      </c>
+      <c r="F340" t="n">
+        <v>0</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
+      <c r="H340" t="n">
+        <v>0</v>
+      </c>
+      <c r="I340" t="n">
+        <v>0</v>
+      </c>
+      <c r="J340" t="n">
+        <v>0</v>
+      </c>
+      <c r="K340" t="n">
+        <v>0</v>
+      </c>
+      <c r="L340" t="n">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>